<commit_message>
fix(catalogs): khac phuc triet de loi khong nap du lieu cu khi hieu chinh hoat dong
</commit_message>
<xml_diff>
--- a/Bao_Cao_Khao_Sat_Dau_Nam_va_76_HS_CKDV_2026.xlsx
+++ b/Bao_Cao_Khao_Sat_Dau_Nam_va_76_HS_CKDV_2026.xlsx
@@ -7177,13 +7177,13 @@
         <v>CS2</v>
       </c>
       <c r="C5" t="str">
-        <v>HS065</v>
+        <v>0601021777</v>
       </c>
       <c r="D5" t="str">
         <v>Lê Gia Lân</v>
       </c>
       <c r="E5" t="str">
-        <v>Chưa rõ</v>
+        <v>1.3_CS2</v>
       </c>
       <c r="F5" t="str">
         <v>Khối 1</v>
@@ -7212,13 +7212,13 @@
         <v>CS2</v>
       </c>
       <c r="C6" t="str">
-        <v>HS079</v>
+        <v>0601021457</v>
       </c>
       <c r="D6" t="str">
         <v>Đào Trần Thảo Linh</v>
       </c>
       <c r="E6" t="str">
-        <v>Chưa rõ</v>
+        <v>1.3_CS2</v>
       </c>
       <c r="F6" t="str">
         <v>Khối 1</v>
@@ -7247,7 +7247,7 @@
         <v>CS1</v>
       </c>
       <c r="C7" t="str">
-        <v>HS105</v>
+        <v>0601011426</v>
       </c>
       <c r="D7" t="str">
         <v>Lê Nguyên Khang</v>
@@ -7282,7 +7282,7 @@
         <v>CS3</v>
       </c>
       <c r="C8" t="str">
-        <v>HS148</v>
+        <v>0701030370</v>
       </c>
       <c r="D8" t="str">
         <v>Phan Anh Quân</v>
@@ -7317,7 +7317,7 @@
         <v>CS3</v>
       </c>
       <c r="C9" t="str">
-        <v>HS163</v>
+        <v>0701030387</v>
       </c>
       <c r="D9" t="str">
         <v>Đoàn Ngọc Thảo Chloe</v>
@@ -7352,7 +7352,7 @@
         <v>CS1</v>
       </c>
       <c r="C10" t="str">
-        <v>HS249</v>
+        <v>0601011201</v>
       </c>
       <c r="D10" t="str">
         <v>Mai Huy Thắng</v>
@@ -7387,7 +7387,7 @@
         <v>CS1</v>
       </c>
       <c r="C11" t="str">
-        <v>HS288</v>
+        <v>0601012396</v>
       </c>
       <c r="D11" t="str">
         <v xml:space="preserve">Trần Hoàng Anh </v>
@@ -7422,7 +7422,7 @@
         <v>CS1</v>
       </c>
       <c r="C12" t="str">
-        <v>HS307</v>
+        <v>0601012393</v>
       </c>
       <c r="D12" t="str">
         <v>Nguyễn Thanh Thảo</v>
@@ -7457,7 +7457,7 @@
         <v>CS1</v>
       </c>
       <c r="C13" t="str">
-        <v>HS308</v>
+        <v>0601011617</v>
       </c>
       <c r="D13" t="str">
         <v>Lê Khánh Hà</v>
@@ -7492,7 +7492,7 @@
         <v>CS1</v>
       </c>
       <c r="C14" t="str">
-        <v>HS701020014</v>
+        <v>0601012399</v>
       </c>
       <c r="D14" t="str">
         <v>Ngô Thục Đan</v>
@@ -7527,13 +7527,13 @@
         <v>CS2</v>
       </c>
       <c r="C15" t="str">
-        <v>HS701020036</v>
+        <v>0601021828</v>
       </c>
       <c r="D15" t="str">
         <v>Phan Hải Đăng</v>
       </c>
       <c r="E15" t="str">
-        <v>Chưa rõ</v>
+        <v>1.3_CS2</v>
       </c>
       <c r="F15" t="str">
         <v>Khối 1</v>
@@ -7562,13 +7562,13 @@
         <v>CS3</v>
       </c>
       <c r="C16" t="str">
-        <v>HS701020076</v>
+        <v>0701030397</v>
       </c>
       <c r="D16" t="str">
         <v>Govorushko Mikhail</v>
       </c>
       <c r="E16" t="str">
-        <v>Chưa rõ</v>
+        <v>1.1INT_CS3</v>
       </c>
       <c r="F16" t="str">
         <v>Khối 1</v>
@@ -7597,7 +7597,7 @@
         <v>CS3</v>
       </c>
       <c r="C17" t="str">
-        <v>HS701020085</v>
+        <v>0701030402</v>
       </c>
       <c r="D17" t="str">
         <v>Lecomte Mailys Mộc Yên</v>
@@ -7632,7 +7632,7 @@
         <v>CS4</v>
       </c>
       <c r="C18" t="str">
-        <v>HS202</v>
+        <v>0602040621</v>
       </c>
       <c r="D18" t="str">
         <v>Võ Thị Anh Thư</v>
@@ -7667,13 +7667,13 @@
         <v>CS2</v>
       </c>
       <c r="C19" t="str">
-        <v>HS701020105</v>
+        <v>0601021795</v>
       </c>
       <c r="D19" t="str">
         <v>Lê Hồ Duy Khang</v>
       </c>
       <c r="E19" t="str">
-        <v>Chưa rõ</v>
+        <v>1.3_CS2</v>
       </c>
       <c r="F19" t="str">
         <v>Khối 1</v>
@@ -7702,13 +7702,13 @@
         <v>CS1</v>
       </c>
       <c r="C20" t="str">
-        <v>HS701020134</v>
+        <v>0601012303</v>
       </c>
       <c r="D20" t="str">
         <v>Nguyễn Daniil</v>
       </c>
       <c r="E20" t="str">
-        <v>Chưa rõ</v>
+        <v>1.1_CS1</v>
       </c>
       <c r="F20" t="str">
         <v>Khối 1</v>
@@ -7737,7 +7737,7 @@
         <v>CS1</v>
       </c>
       <c r="C21" t="str">
-        <v>HS701020183</v>
+        <v>0601012153</v>
       </c>
       <c r="D21" t="str">
         <v>Nguyễn Ngọc Minh</v>
@@ -7772,13 +7772,13 @@
         <v>CS2</v>
       </c>
       <c r="C22" t="str">
-        <v>HS701020188</v>
+        <v>0701020109</v>
       </c>
       <c r="D22" t="str">
         <v>Sangadziev Aron</v>
       </c>
       <c r="E22" t="str">
-        <v>Chưa rõ</v>
+        <v>1.2INT_CS2</v>
       </c>
       <c r="F22" t="str">
         <v>Khối 1</v>
@@ -7868,7 +7868,7 @@
         <v>CS1</v>
       </c>
       <c r="C6" t="str">
-        <v>HS101</v>
+        <v>0701030312</v>
       </c>
       <c r="D6" t="str">
         <v>Nguyễn Gia Bảo</v>
@@ -7903,7 +7903,7 @@
         <v>CS1</v>
       </c>
       <c r="C7" t="str">
-        <v>HS105</v>
+        <v>0601011426</v>
       </c>
       <c r="D7" t="str">
         <v>Lê Nguyên Khang</v>
@@ -7938,7 +7938,7 @@
         <v>CS1</v>
       </c>
       <c r="C8" t="str">
-        <v>HS111</v>
+        <v>0601012314</v>
       </c>
       <c r="D8" t="str">
         <v>Phạm Nguyễn Minh Anh</v>
@@ -7973,7 +7973,7 @@
         <v>CS1</v>
       </c>
       <c r="C9" t="str">
-        <v>HS246</v>
+        <v>0601012372</v>
       </c>
       <c r="D9" t="str">
         <v>Phan Đình Phùng</v>
@@ -8008,7 +8008,7 @@
         <v>CS1</v>
       </c>
       <c r="C10" t="str">
-        <v>HS249</v>
+        <v>0601011201</v>
       </c>
       <c r="D10" t="str">
         <v>Mai Huy Thắng</v>
@@ -8043,7 +8043,7 @@
         <v>CS1</v>
       </c>
       <c r="C11" t="str">
-        <v>HS252</v>
+        <v>0601012363</v>
       </c>
       <c r="D11" t="str">
         <v xml:space="preserve">Phạm Thùy Gia Hân </v>
@@ -8078,7 +8078,7 @@
         <v>CS1</v>
       </c>
       <c r="C12" t="str">
-        <v>HS256</v>
+        <v>0601012381</v>
       </c>
       <c r="D12" t="str">
         <v>Nguyễn Bình Phương An</v>
@@ -8113,7 +8113,7 @@
         <v>CS1</v>
       </c>
       <c r="C13" t="str">
-        <v>HS257</v>
+        <v>0601050347</v>
       </c>
       <c r="D13" t="str">
         <v>Lê Bảo Trâm</v>
@@ -8148,7 +8148,7 @@
         <v>CS1</v>
       </c>
       <c r="C14" t="str">
-        <v>HS258</v>
+        <v>0601011593</v>
       </c>
       <c r="D14" t="str">
         <v>Lê Bảo Châu</v>
@@ -8183,7 +8183,7 @@
         <v>CS1</v>
       </c>
       <c r="C15" t="str">
-        <v>HS259</v>
+        <v>0601012376</v>
       </c>
       <c r="D15" t="str">
         <v>Phạm Gia Hương</v>
@@ -8218,13 +8218,13 @@
         <v>CS1</v>
       </c>
       <c r="C16" t="str">
-        <v>HS265</v>
+        <v>0601012390</v>
       </c>
       <c r="D16" t="str">
         <v xml:space="preserve">Đỗ An Nhiên </v>
       </c>
       <c r="E16" t="str">
-        <v>Chưa rõ</v>
+        <v>1.1_CS1</v>
       </c>
       <c r="F16" t="str">
         <v>Khối 1</v>
@@ -8253,13 +8253,13 @@
         <v>CS1</v>
       </c>
       <c r="C17" t="str">
-        <v>HS275</v>
+        <v>0602040631</v>
       </c>
       <c r="D17" t="str">
         <v>Hà Đặng Phước Huy</v>
       </c>
       <c r="E17" t="str">
-        <v>Chưa rõ</v>
+        <v>1S_CS4</v>
       </c>
       <c r="F17" t="str">
         <v>Khối 1</v>
@@ -8288,7 +8288,7 @@
         <v>CS1</v>
       </c>
       <c r="C18" t="str">
-        <v>HS288</v>
+        <v>0601012396</v>
       </c>
       <c r="D18" t="str">
         <v xml:space="preserve">Trần Hoàng Anh </v>
@@ -8323,7 +8323,7 @@
         <v>CS1</v>
       </c>
       <c r="C19" t="str">
-        <v>HS306</v>
+        <v>0701010055</v>
       </c>
       <c r="D19" t="str">
         <v>Nguyễn Ngọc Thiên Bảo</v>
@@ -8358,7 +8358,7 @@
         <v>CS1</v>
       </c>
       <c r="C20" t="str">
-        <v>HS307</v>
+        <v>0601012393</v>
       </c>
       <c r="D20" t="str">
         <v>Nguyễn Thanh Thảo</v>
@@ -8393,7 +8393,7 @@
         <v>CS1</v>
       </c>
       <c r="C21" t="str">
-        <v>HS308</v>
+        <v>0601011617</v>
       </c>
       <c r="D21" t="str">
         <v>Lê Khánh Hà</v>
@@ -8428,7 +8428,7 @@
         <v>CS1</v>
       </c>
       <c r="C22" t="str">
-        <v>HS311</v>
+        <v>0601012394</v>
       </c>
       <c r="D22" t="str">
         <v xml:space="preserve">Nguyễn Đại Phúc </v>
@@ -8469,7 +8469,7 @@
         <v>LÊ ĐÌNH SĨ PHÚ</v>
       </c>
       <c r="E23" t="str">
-        <v>Chưa rõ</v>
+        <v>6.1_CS1</v>
       </c>
       <c r="F23" t="str">
         <v>Khối 6</v>
@@ -8498,7 +8498,7 @@
         <v>CS1</v>
       </c>
       <c r="C24" t="str">
-        <v>HS701020014</v>
+        <v>0601012399</v>
       </c>
       <c r="D24" t="str">
         <v>Ngô Thục Đan</v>
@@ -8533,7 +8533,7 @@
         <v>CS1</v>
       </c>
       <c r="C25" t="str">
-        <v>HS116</v>
+        <v>0601012317</v>
       </c>
       <c r="D25" t="str">
         <v>Lê Nguyệt Cát</v>
@@ -8568,7 +8568,7 @@
         <v>CS1</v>
       </c>
       <c r="C26" t="str">
-        <v>HS129</v>
+        <v>0601012338</v>
       </c>
       <c r="D26" t="str">
         <v>Hoàng Bảo Quyên</v>
@@ -8603,7 +8603,7 @@
         <v>CS1</v>
       </c>
       <c r="C27" t="str">
-        <v>HS131</v>
+        <v>0601012280</v>
       </c>
       <c r="D27" t="str">
         <v>Phạm Gia Bảo</v>
@@ -8638,7 +8638,7 @@
         <v>CS1</v>
       </c>
       <c r="C28" t="str">
-        <v>HS124</v>
+        <v>0601012318</v>
       </c>
       <c r="D28" t="str">
         <v>Đặng Hoàng Như Ý</v>
@@ -8673,7 +8673,7 @@
         <v>CS1</v>
       </c>
       <c r="C29" t="str">
-        <v>HS126</v>
+        <v>0601012334</v>
       </c>
       <c r="D29" t="str">
         <v>Phạm Hải Như</v>
@@ -8708,7 +8708,7 @@
         <v>CS1</v>
       </c>
       <c r="C30" t="str">
-        <v>HS701020117</v>
+        <v>0701030403</v>
       </c>
       <c r="D30" t="str">
         <v>Nguyễn Thành Long</v>
@@ -8743,7 +8743,7 @@
         <v>CS1</v>
       </c>
       <c r="C31" t="str">
-        <v>HS701020124</v>
+        <v>0601012369</v>
       </c>
       <c r="D31" t="str">
         <v>Trần Quang Thiên Ân</v>
@@ -8778,7 +8778,7 @@
         <v>CS1</v>
       </c>
       <c r="C32" t="str">
-        <v>HS701020125</v>
+        <v>0601012312</v>
       </c>
       <c r="D32" t="str">
         <v>Lê Hồ Gia Huy</v>
@@ -8813,7 +8813,7 @@
         <v>CS1</v>
       </c>
       <c r="C33" t="str">
-        <v>HS701020126</v>
+        <v>0601012400</v>
       </c>
       <c r="D33" t="str">
         <v>Trương Lê Hưng Phát</v>
@@ -8848,7 +8848,7 @@
         <v>CS1</v>
       </c>
       <c r="C34" t="str">
-        <v>HS701020122</v>
+        <v>0601012351</v>
       </c>
       <c r="D34" t="str">
         <v>Nguyễn Văn Tuấn Kiệt</v>
@@ -8883,13 +8883,13 @@
         <v>CS1</v>
       </c>
       <c r="C35" t="str">
-        <v>HS701020134</v>
+        <v>0601012303</v>
       </c>
       <c r="D35" t="str">
         <v>Nguyễn Daniil</v>
       </c>
       <c r="E35" t="str">
-        <v>Chưa rõ</v>
+        <v>1.1_CS1</v>
       </c>
       <c r="F35" t="str">
         <v>Khối 1</v>
@@ -8918,7 +8918,7 @@
         <v>CS1</v>
       </c>
       <c r="C36" t="str">
-        <v>HS701020137</v>
+        <v>0601012340</v>
       </c>
       <c r="D36" t="str">
         <v>Trần Đăng Quang</v>
@@ -8953,7 +8953,7 @@
         <v>CS1</v>
       </c>
       <c r="C37" t="str">
-        <v>HS701020139</v>
+        <v>0601012347</v>
       </c>
       <c r="D37" t="str">
         <v>Trần Thục Quyên</v>
@@ -8988,7 +8988,7 @@
         <v>CS1</v>
       </c>
       <c r="C38" t="str">
-        <v>HS701020140</v>
+        <v>0601012348</v>
       </c>
       <c r="D38" t="str">
         <v>Lương Bích Ngọc</v>
@@ -9023,7 +9023,7 @@
         <v>CS1</v>
       </c>
       <c r="C39" t="str">
-        <v>HS701020141</v>
+        <v>0601011972</v>
       </c>
       <c r="D39" t="str">
         <v>Nguyễn Quỳnh Như</v>
@@ -9058,7 +9058,7 @@
         <v>CS1</v>
       </c>
       <c r="C40" t="str">
-        <v>HS701020183</v>
+        <v>0601012153</v>
       </c>
       <c r="D40" t="str">
         <v>Nguyễn Ngọc Minh</v>
@@ -9093,7 +9093,7 @@
         <v>CS1</v>
       </c>
       <c r="C41" t="str">
-        <v>HS701020186</v>
+        <v>0601012421</v>
       </c>
       <c r="D41" t="str">
         <v xml:space="preserve">Nguyễn Đặng Bảo Trâm </v>
@@ -9128,13 +9128,13 @@
         <v>CS2</v>
       </c>
       <c r="C42" t="str">
-        <v>HS065</v>
+        <v>0601021777</v>
       </c>
       <c r="D42" t="str">
         <v>Lê Gia Lân</v>
       </c>
       <c r="E42" t="str">
-        <v>Chưa rõ</v>
+        <v>1.3_CS2</v>
       </c>
       <c r="F42" t="str">
         <v>Khối 1</v>
@@ -9163,13 +9163,13 @@
         <v>CS2</v>
       </c>
       <c r="C43" t="str">
-        <v>HS079</v>
+        <v>0601021457</v>
       </c>
       <c r="D43" t="str">
         <v>Đào Trần Thảo Linh</v>
       </c>
       <c r="E43" t="str">
-        <v>Chưa rõ</v>
+        <v>1.3_CS2</v>
       </c>
       <c r="F43" t="str">
         <v>Khối 1</v>
@@ -9198,13 +9198,13 @@
         <v>CS2</v>
       </c>
       <c r="C44" t="str">
-        <v>HS083</v>
+        <v>0701020104</v>
       </c>
       <c r="D44" t="str">
         <v>Nguyễn Thanh Phúc</v>
       </c>
       <c r="E44" t="str">
-        <v>Chưa rõ</v>
+        <v>1.2INT_CS2</v>
       </c>
       <c r="F44" t="str">
         <v>Khối 1</v>
@@ -9233,13 +9233,13 @@
         <v>CS2</v>
       </c>
       <c r="C45" t="str">
-        <v>HS286</v>
+        <v>0601021794</v>
       </c>
       <c r="D45" t="str">
         <v>ĐỖ NGUYỄN AN KHÔI</v>
       </c>
       <c r="E45" t="str">
-        <v>Chưa rõ</v>
+        <v>1.3_CS2</v>
       </c>
       <c r="F45" t="str">
         <v>Khối 1</v>
@@ -9268,13 +9268,13 @@
         <v>CS2</v>
       </c>
       <c r="C46" t="str">
-        <v>HS701020036</v>
+        <v>0601021828</v>
       </c>
       <c r="D46" t="str">
         <v>Phan Hải Đăng</v>
       </c>
       <c r="E46" t="str">
-        <v>Chưa rõ</v>
+        <v>1.3_CS2</v>
       </c>
       <c r="F46" t="str">
         <v>Khối 1</v>
@@ -9303,7 +9303,7 @@
         <v>CS2</v>
       </c>
       <c r="C47" t="str">
-        <v>HS701020095</v>
+        <v>0601012037</v>
       </c>
       <c r="D47" t="str">
         <v>Hoàng Bữu Minh Hưng</v>
@@ -9338,13 +9338,13 @@
         <v>CS2</v>
       </c>
       <c r="C48" t="str">
-        <v>HS701020105</v>
+        <v>0601021795</v>
       </c>
       <c r="D48" t="str">
         <v>Lê Hồ Duy Khang</v>
       </c>
       <c r="E48" t="str">
-        <v>Chưa rõ</v>
+        <v>1.3_CS2</v>
       </c>
       <c r="F48" t="str">
         <v>Khối 1</v>
@@ -9373,13 +9373,13 @@
         <v>CS2</v>
       </c>
       <c r="C49" t="str">
-        <v>HS701020188</v>
+        <v>0701020109</v>
       </c>
       <c r="D49" t="str">
         <v>Sangadziev Aron</v>
       </c>
       <c r="E49" t="str">
-        <v>Chưa rõ</v>
+        <v>1.2INT_CS2</v>
       </c>
       <c r="F49" t="str">
         <v>Khối 1</v>
@@ -9408,7 +9408,7 @@
         <v>CS3</v>
       </c>
       <c r="C50" t="str">
-        <v>HS148</v>
+        <v>0701030370</v>
       </c>
       <c r="D50" t="str">
         <v>Phan Anh Quân</v>
@@ -9443,7 +9443,7 @@
         <v>CS3</v>
       </c>
       <c r="C51" t="str">
-        <v>HS163</v>
+        <v>0701030387</v>
       </c>
       <c r="D51" t="str">
         <v>Đoàn Ngọc Thảo Chloe</v>
@@ -9478,7 +9478,7 @@
         <v>CS3</v>
       </c>
       <c r="C52" t="str">
-        <v>HS175</v>
+        <v>0501030625</v>
       </c>
       <c r="D52" t="str">
         <v>Hồ Hữu Bách</v>
@@ -9513,13 +9513,13 @@
         <v>CS3</v>
       </c>
       <c r="C53" t="str">
-        <v>HS701020076</v>
+        <v>0701030397</v>
       </c>
       <c r="D53" t="str">
         <v>Govorushko Mikhail</v>
       </c>
       <c r="E53" t="str">
-        <v>Chưa rõ</v>
+        <v>1.1INT_CS3</v>
       </c>
       <c r="F53" t="str">
         <v>Khối 1</v>
@@ -9548,7 +9548,7 @@
         <v>CS3</v>
       </c>
       <c r="C54" t="str">
-        <v>HS701020085</v>
+        <v>0701030402</v>
       </c>
       <c r="D54" t="str">
         <v>Lecomte Mailys Mộc Yên</v>
@@ -9583,7 +9583,7 @@
         <v>CS3</v>
       </c>
       <c r="C55" t="str">
-        <v>HS701020094</v>
+        <v>0701030384</v>
       </c>
       <c r="D55" t="str">
         <v>Hà Minh Khuê</v>
@@ -9618,7 +9618,7 @@
         <v>CS3</v>
       </c>
       <c r="C56" t="str">
-        <v>HS701020184</v>
+        <v>0701030415</v>
       </c>
       <c r="D56" t="str">
         <v>Phùng Đức Thiên Ân</v>
@@ -9653,7 +9653,7 @@
         <v>CS3</v>
       </c>
       <c r="C57" t="str">
-        <v>HS701020185</v>
+        <v>0701030416</v>
       </c>
       <c r="D57" t="str">
         <v>Phùng Chí Nam Anh</v>
@@ -9688,7 +9688,7 @@
         <v>CS4</v>
       </c>
       <c r="C58" t="str">
-        <v>HS179</v>
+        <v>0602040593</v>
       </c>
       <c r="D58" t="str">
         <v>Ayesha Mirza</v>
@@ -9723,7 +9723,7 @@
         <v>CS4</v>
       </c>
       <c r="C59" t="str">
-        <v>HS276</v>
+        <v>0602040630</v>
       </c>
       <c r="D59" t="str">
         <v>HÀ ĐẶNG BẢO NGỌC</v>
@@ -9758,7 +9758,7 @@
         <v>CS4</v>
       </c>
       <c r="C60" t="str">
-        <v>HS283</v>
+        <v>0601012397</v>
       </c>
       <c r="D60" t="str">
         <v>Nguyễn Thị Thu Thúy</v>
@@ -9793,7 +9793,7 @@
         <v>CS4</v>
       </c>
       <c r="C61" t="str">
-        <v>HS293</v>
+        <v>0602040636</v>
       </c>
       <c r="D61" t="str">
         <v>Huỳnh Hoàng An</v>
@@ -9828,7 +9828,7 @@
         <v>CS4</v>
       </c>
       <c r="C62" t="str">
-        <v>HS701020029</v>
+        <v>0602040624</v>
       </c>
       <c r="D62" t="str">
         <v>Đặng Ngọc Bảo Ngân</v>
@@ -9863,7 +9863,7 @@
         <v>CS4</v>
       </c>
       <c r="C63" t="str">
-        <v>HS701020030</v>
+        <v>0602040623</v>
       </c>
       <c r="D63" t="str">
         <v>Ngô Nhật Khang</v>
@@ -9898,7 +9898,7 @@
         <v>CS4</v>
       </c>
       <c r="C64" t="str">
-        <v>HS701020033</v>
+        <v>0602040522</v>
       </c>
       <c r="D64" t="str">
         <v>Võ Hoàng Vi</v>
@@ -9933,7 +9933,7 @@
         <v>CS4</v>
       </c>
       <c r="C65" t="str">
-        <v>HS701020061</v>
+        <v>0602040642</v>
       </c>
       <c r="D65" t="str">
         <v>Võ Như Quỳnh</v>
@@ -9968,7 +9968,7 @@
         <v>CS4</v>
       </c>
       <c r="C66" t="str">
-        <v>HS701020064</v>
+        <v>0602040613</v>
       </c>
       <c r="D66" t="str">
         <v>Đỗ Thành Nguyên</v>
@@ -10003,7 +10003,7 @@
         <v>CS4</v>
       </c>
       <c r="C67" t="str">
-        <v>HS701020065</v>
+        <v>0602040586</v>
       </c>
       <c r="D67" t="str">
         <v>Phạm Kiều Anh</v>
@@ -10038,7 +10038,7 @@
         <v>CS4</v>
       </c>
       <c r="C68" t="str">
-        <v>HS202</v>
+        <v>0602040621</v>
       </c>
       <c r="D68" t="str">
         <v>Võ Thị Anh Thư</v>
@@ -10073,13 +10073,13 @@
         <v>CS4</v>
       </c>
       <c r="C69" t="str">
-        <v>HS701020195</v>
+        <v>0602040655</v>
       </c>
       <c r="D69" t="str">
         <v>Ngô Huỳnh Anh Minh</v>
       </c>
       <c r="E69" t="str">
-        <v>Chưa rõ</v>
+        <v>6S_CS4</v>
       </c>
       <c r="F69" t="str">
         <v>Khối 6</v>
@@ -10108,7 +10108,7 @@
         <v>CS5</v>
       </c>
       <c r="C70" t="str">
-        <v>HS218</v>
+        <v>0601051095</v>
       </c>
       <c r="D70" t="str">
         <v>Mai Minh Minh</v>
@@ -10143,7 +10143,7 @@
         <v>CS5</v>
       </c>
       <c r="C71" t="str">
-        <v>HS240</v>
+        <v>0601051137</v>
       </c>
       <c r="D71" t="str">
         <v>Lâm Minh Khang</v>
@@ -10178,7 +10178,7 @@
         <v>CS5</v>
       </c>
       <c r="C72" t="str">
-        <v>HS334</v>
+        <v>0601051161</v>
       </c>
       <c r="D72" t="str">
         <v>Đặng Ái Thiên Vân</v>
@@ -10248,7 +10248,7 @@
         <v>CS5</v>
       </c>
       <c r="C74" t="str">
-        <v>HS132</v>
+        <v>0701030326</v>
       </c>
       <c r="D74" t="str">
         <v>Phạm Gia Hưng</v>
@@ -10283,13 +10283,13 @@
         <v>CS5</v>
       </c>
       <c r="C75" t="str">
-        <v>HS701020154</v>
+        <v>0601051050</v>
       </c>
       <c r="D75" t="str">
         <v>Vũ Đức Thịnh</v>
       </c>
       <c r="E75" t="str">
-        <v>Chưa rõ</v>
+        <v>1.5_CS5</v>
       </c>
       <c r="F75" t="str">
         <v>Khối 1</v>
@@ -10318,7 +10318,7 @@
         <v>CS5</v>
       </c>
       <c r="C76" t="str">
-        <v>HS701020159</v>
+        <v>0501030605</v>
       </c>
       <c r="D76" t="str">
         <v>Nguyễn Minh Anh</v>
@@ -10353,7 +10353,7 @@
         <v>CS5</v>
       </c>
       <c r="C77" t="str">
-        <v>HS701020158</v>
+        <v>0601051037</v>
       </c>
       <c r="D77" t="str">
         <v>Đỗ Duy Khôi</v>
@@ -10388,7 +10388,7 @@
         <v>CS5</v>
       </c>
       <c r="C78" t="str">
-        <v>HS701020163</v>
+        <v>0601051152</v>
       </c>
       <c r="D78" t="str">
         <v>Lê Nguyễn Hoàng Bảo</v>
@@ -10423,7 +10423,7 @@
         <v>CS5</v>
       </c>
       <c r="C79" t="str">
-        <v>HS701020167</v>
+        <v>0701050069</v>
       </c>
       <c r="D79" t="str">
         <v>Nguyễn Hoàng Đạt</v>
@@ -10458,7 +10458,7 @@
         <v>CS5</v>
       </c>
       <c r="C80" t="str">
-        <v>HS701020170</v>
+        <v>0701050068</v>
       </c>
       <c r="D80" t="str">
         <v>Nguyễn Hoàng Phúc</v>
@@ -10493,7 +10493,7 @@
         <v>CS5</v>
       </c>
       <c r="C81" t="str">
-        <v>HS701020166</v>
+        <v>0701030411</v>
       </c>
       <c r="D81" t="str">
         <v>Trần Minh Huy</v>

</xml_diff>

<commit_message>
feat(experiential): dong bo hien thi tat ca hoat dong tu ca Danh muc va Trien khai, bo sung menu sidebar
</commit_message>
<xml_diff>
--- a/Bao_Cao_Khao_Sat_Dau_Nam_va_76_HS_CKDV_2026.xlsx
+++ b/Bao_Cao_Khao_Sat_Dau_Nam_va_76_HS_CKDV_2026.xlsx
@@ -7,9 +7,8 @@
     <sheet name="Tieu_Hoc_Theo_CS" sheetId="2" r:id="rId2"/>
     <sheet name="THCS_Theo_CS" sheetId="3" r:id="rId3"/>
     <sheet name="THPT_Theo_CS" sheetId="4" r:id="rId4"/>
-    <sheet name="THPT_7_Mon_Tu_Chon_K12" sheetId="5" r:id="rId5"/>
-    <sheet name="HS_Chua_Du_Diem_KSDV" sheetId="6" r:id="rId6"/>
-    <sheet name="76_HS_CKDV" sheetId="7" r:id="rId7"/>
+    <sheet name="HS_Chua_Du_Diem_KSDV" sheetId="5" r:id="rId5"/>
+    <sheet name="76_HS_CKDV" sheetId="6" r:id="rId6"/>
   </sheets>
 </workbook>
 </file>
@@ -484,10 +483,10 @@
         <v>89.0%</v>
       </c>
       <c r="I6">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="J6" t="str">
-        <v>2.0%</v>
+        <v>1.9%</v>
       </c>
       <c r="K6">
         <v>2002</v>
@@ -522,10 +521,10 @@
         <v>85.2%</v>
       </c>
       <c r="I7">
-        <v>310</v>
+        <v>243</v>
       </c>
       <c r="J7" t="str">
-        <v>14.8%</v>
+        <v>11.6%</v>
       </c>
       <c r="K7">
         <v>838</v>
@@ -560,10 +559,10 @@
         <v>65.7%</v>
       </c>
       <c r="I8">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="J8" t="str">
-        <v>34.3%</v>
+        <v>33.9%</v>
       </c>
       <c r="K8">
         <v>76</v>
@@ -598,10 +597,10 @@
         <v>85.2%</v>
       </c>
       <c r="I9">
-        <v>537</v>
+        <v>464</v>
       </c>
       <c r="J9" t="str">
-        <v>10.3%</v>
+        <v>8.9%</v>
       </c>
       <c r="K9">
         <v>2916</v>
@@ -1126,10 +1125,10 @@
         <v>57</v>
       </c>
       <c r="E13">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F13" t="str">
-        <v>3.5%</v>
+        <v>1.8%</v>
       </c>
       <c r="G13">
         <v>53</v>
@@ -1158,10 +1157,10 @@
         <v>60</v>
       </c>
       <c r="E14">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F14" t="str">
-        <v>3.3%</v>
+        <v>1.7%</v>
       </c>
       <c r="G14">
         <v>53</v>
@@ -1350,10 +1349,10 @@
         <v>720</v>
       </c>
       <c r="E20">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="F20" t="str">
-        <v>1.8%</v>
+        <v>1.5%</v>
       </c>
       <c r="G20">
         <v>646</v>
@@ -2810,10 +2809,10 @@
         <v>44</v>
       </c>
       <c r="E73">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F73" t="str">
-        <v>2.3%</v>
+        <v>0.0%</v>
       </c>
       <c r="G73">
         <v>40</v>
@@ -3130,10 +3129,10 @@
         <v>49</v>
       </c>
       <c r="E83">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F83" t="str">
-        <v>2.0%</v>
+        <v>0.0%</v>
       </c>
       <c r="G83">
         <v>37</v>
@@ -3354,10 +3353,10 @@
         <v>697</v>
       </c>
       <c r="E90">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="F90" t="str">
-        <v>2.2%</v>
+        <v>1.9%</v>
       </c>
       <c r="G90">
         <v>609</v>
@@ -3386,10 +3385,10 @@
         <v>2624</v>
       </c>
       <c r="E92">
-        <v>53</v>
+        <v>49</v>
       </c>
       <c r="F92" t="str">
-        <v>2.0%</v>
+        <v>1.9%</v>
       </c>
       <c r="G92">
         <v>2335</v>
@@ -3482,10 +3481,10 @@
         <v>2.8%</v>
       </c>
       <c r="G6">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="H6" t="str">
-        <v>94.4%</v>
+        <v>97.2%</v>
       </c>
       <c r="I6">
         <v>45</v>
@@ -3508,16 +3507,16 @@
         <v>99</v>
       </c>
       <c r="E7">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F7" t="str">
-        <v>3.0%</v>
+        <v>2.0%</v>
       </c>
       <c r="G7">
-        <v>89</v>
+        <v>96</v>
       </c>
       <c r="H7" t="str">
-        <v>89.9%</v>
+        <v>97.0%</v>
       </c>
       <c r="I7">
         <v>68</v>
@@ -3546,10 +3545,10 @@
         <v>37.5%</v>
       </c>
       <c r="G8">
-        <v>25</v>
+        <v>40</v>
       </c>
       <c r="H8" t="str">
-        <v>39.1%</v>
+        <v>62.5%</v>
       </c>
       <c r="I8">
         <v>3</v>
@@ -3578,10 +3577,10 @@
         <v>14.7%</v>
       </c>
       <c r="G9">
-        <v>75</v>
+        <v>87</v>
       </c>
       <c r="H9" t="str">
-        <v>73.5%</v>
+        <v>85.3%</v>
       </c>
       <c r="I9">
         <v>50</v>
@@ -3610,10 +3609,10 @@
         <v>1.4%</v>
       </c>
       <c r="G10">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="H10" t="str">
-        <v>95.8%</v>
+        <v>98.6%</v>
       </c>
       <c r="I10">
         <v>37</v>
@@ -3642,10 +3641,10 @@
         <v>10.2%</v>
       </c>
       <c r="G11">
-        <v>78</v>
+        <v>88</v>
       </c>
       <c r="H11" t="str">
-        <v>79.6%</v>
+        <v>89.8%</v>
       </c>
       <c r="I11">
         <v>35</v>
@@ -3674,10 +3673,10 @@
         <v>1.5%</v>
       </c>
       <c r="G12">
-        <v>57</v>
+        <v>64</v>
       </c>
       <c r="H12" t="str">
-        <v>87.7%</v>
+        <v>98.5%</v>
       </c>
       <c r="I12">
         <v>27</v>
@@ -3706,10 +3705,10 @@
         <v>16.8%</v>
       </c>
       <c r="G13">
-        <v>73</v>
+        <v>84</v>
       </c>
       <c r="H13" t="str">
-        <v>72.3%</v>
+        <v>83.2%</v>
       </c>
       <c r="I13">
         <v>28</v>
@@ -3738,10 +3737,10 @@
         <v>6.9%</v>
       </c>
       <c r="G14">
-        <v>59</v>
+        <v>67</v>
       </c>
       <c r="H14" t="str">
-        <v>81.9%</v>
+        <v>93.1%</v>
       </c>
       <c r="I14">
         <v>44</v>
@@ -3770,10 +3769,10 @@
         <v>13.4%</v>
       </c>
       <c r="G15">
-        <v>73</v>
+        <v>84</v>
       </c>
       <c r="H15" t="str">
-        <v>75.3%</v>
+        <v>86.6%</v>
       </c>
       <c r="I15">
         <v>40</v>
@@ -3802,10 +3801,10 @@
         <v>15.6%</v>
       </c>
       <c r="G16">
-        <v>45</v>
+        <v>54</v>
       </c>
       <c r="H16" t="str">
-        <v>70.3%</v>
+        <v>84.4%</v>
       </c>
       <c r="I16">
         <v>19</v>
@@ -3834,10 +3833,10 @@
         <v>12.7%</v>
       </c>
       <c r="G17">
-        <v>84</v>
+        <v>89</v>
       </c>
       <c r="H17" t="str">
-        <v>82.4%</v>
+        <v>87.3%</v>
       </c>
       <c r="I17">
         <v>55</v>
@@ -3860,16 +3859,16 @@
         <v>1008</v>
       </c>
       <c r="E18">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="F18" t="str">
-        <v>11.3%</v>
+        <v>11.2%</v>
       </c>
       <c r="G18">
-        <v>795</v>
+        <v>894</v>
       </c>
       <c r="H18" t="str">
-        <v>78.9%</v>
+        <v>88.7%</v>
       </c>
       <c r="I18">
         <v>451</v>
@@ -3929,10 +3928,10 @@
         <v>39</v>
       </c>
       <c r="E22">
-        <v>21</v>
+        <v>1</v>
       </c>
       <c r="F22" t="str">
-        <v>53.8%</v>
+        <v>2.6%</v>
       </c>
       <c r="G22">
         <v>18</v>
@@ -3961,10 +3960,10 @@
         <v>46</v>
       </c>
       <c r="E23">
-        <v>46</v>
+        <v>0</v>
       </c>
       <c r="F23" t="str">
-        <v>100.0%</v>
+        <v>0.0%</v>
       </c>
       <c r="G23">
         <v>0</v>
@@ -3999,10 +3998,10 @@
         <v>18.2%</v>
       </c>
       <c r="G24">
-        <v>22</v>
+        <v>27</v>
       </c>
       <c r="H24" t="str">
-        <v>66.7%</v>
+        <v>81.8%</v>
       </c>
       <c r="I24">
         <v>5</v>
@@ -4031,10 +4030,10 @@
         <v>15.0%</v>
       </c>
       <c r="G25">
-        <v>18</v>
+        <v>34</v>
       </c>
       <c r="H25" t="str">
-        <v>45.0%</v>
+        <v>85.0%</v>
       </c>
       <c r="I25">
         <v>7</v>
@@ -4063,10 +4062,10 @@
         <v>2.6%</v>
       </c>
       <c r="G26">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="H26" t="str">
-        <v>89.7%</v>
+        <v>97.4%</v>
       </c>
       <c r="I26">
         <v>27</v>
@@ -4095,10 +4094,10 @@
         <v>4.3%</v>
       </c>
       <c r="G27">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="H27" t="str">
-        <v>87.0%</v>
+        <v>95.7%</v>
       </c>
       <c r="I27">
         <v>21</v>
@@ -4159,10 +4158,10 @@
         <v>0.0%</v>
       </c>
       <c r="G29">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="H29" t="str">
-        <v>92.3%</v>
+        <v>100.0%</v>
       </c>
       <c r="I29">
         <v>16</v>
@@ -4191,10 +4190,10 @@
         <v>2.2%</v>
       </c>
       <c r="G30">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="H30" t="str">
-        <v>89.1%</v>
+        <v>97.8%</v>
       </c>
       <c r="I30">
         <v>28</v>
@@ -4223,10 +4222,10 @@
         <v>21.2%</v>
       </c>
       <c r="G31">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="H31" t="str">
-        <v>69.7%</v>
+        <v>78.8%</v>
       </c>
       <c r="I31">
         <v>9</v>
@@ -4255,10 +4254,10 @@
         <v>0.0%</v>
       </c>
       <c r="G32">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="H32" t="str">
-        <v>85.0%</v>
+        <v>100.0%</v>
       </c>
       <c r="I32">
         <v>15</v>
@@ -4319,10 +4318,10 @@
         <v>10.9%</v>
       </c>
       <c r="G34">
-        <v>25</v>
+        <v>41</v>
       </c>
       <c r="H34" t="str">
-        <v>54.3%</v>
+        <v>89.1%</v>
       </c>
       <c r="I34">
         <v>9</v>
@@ -4351,10 +4350,10 @@
         <v>6.1%</v>
       </c>
       <c r="G35">
-        <v>25</v>
+        <v>31</v>
       </c>
       <c r="H35" t="str">
-        <v>75.8%</v>
+        <v>93.9%</v>
       </c>
       <c r="I35">
         <v>11</v>
@@ -4377,16 +4376,16 @@
         <v>559</v>
       </c>
       <c r="E36">
-        <v>97</v>
+        <v>31</v>
       </c>
       <c r="F36" t="str">
-        <v>17.4%</v>
+        <v>5.5%</v>
       </c>
       <c r="G36">
-        <v>396</v>
+        <v>462</v>
       </c>
       <c r="H36" t="str">
-        <v>70.8%</v>
+        <v>82.6%</v>
       </c>
       <c r="I36">
         <v>211</v>
@@ -4452,10 +4451,10 @@
         <v>16.7%</v>
       </c>
       <c r="G40">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="H40" t="str">
-        <v>72.2%</v>
+        <v>83.3%</v>
       </c>
       <c r="I40">
         <v>10</v>
@@ -4516,10 +4515,10 @@
         <v>78.6%</v>
       </c>
       <c r="G42">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H42" t="str">
-        <v>14.3%</v>
+        <v>21.4%</v>
       </c>
       <c r="I42">
         <v>0</v>
@@ -4548,10 +4547,10 @@
         <v>25.0%</v>
       </c>
       <c r="G43">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="H43" t="str">
-        <v>68.8%</v>
+        <v>75.0%</v>
       </c>
       <c r="I43">
         <v>3</v>
@@ -4580,10 +4579,10 @@
         <v>21.1%</v>
       </c>
       <c r="G44">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="H44" t="str">
-        <v>52.6%</v>
+        <v>78.9%</v>
       </c>
       <c r="I44">
         <v>1</v>
@@ -4612,10 +4611,10 @@
         <v>0.0%</v>
       </c>
       <c r="G45">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H45" t="str">
-        <v>90.0%</v>
+        <v>100.0%</v>
       </c>
       <c r="I45">
         <v>5</v>
@@ -4676,10 +4675,10 @@
         <v>37.5%</v>
       </c>
       <c r="G47">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="H47" t="str">
-        <v>31.3%</v>
+        <v>62.5%</v>
       </c>
       <c r="I47">
         <v>2</v>
@@ -4708,10 +4707,10 @@
         <v>42.1%</v>
       </c>
       <c r="G48">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="H48" t="str">
-        <v>52.6%</v>
+        <v>57.9%</v>
       </c>
       <c r="I48">
         <v>1</v>
@@ -4740,10 +4739,10 @@
         <v>30.0%</v>
       </c>
       <c r="G49">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H49" t="str">
-        <v>60.0%</v>
+        <v>70.0%</v>
       </c>
       <c r="I49">
         <v>2</v>
@@ -4772,10 +4771,10 @@
         <v>7.1%</v>
       </c>
       <c r="G50">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="H50" t="str">
-        <v>78.6%</v>
+        <v>92.9%</v>
       </c>
       <c r="I50">
         <v>6</v>
@@ -4804,10 +4803,10 @@
         <v>25.0%</v>
       </c>
       <c r="G51">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="H51" t="str">
-        <v>68.8%</v>
+        <v>75.0%</v>
       </c>
       <c r="I51">
         <v>8</v>
@@ -4836,10 +4835,10 @@
         <v>27.8%</v>
       </c>
       <c r="G52">
-        <v>107</v>
+        <v>127</v>
       </c>
       <c r="H52" t="str">
-        <v>60.8%</v>
+        <v>72.2%</v>
       </c>
       <c r="I52">
         <v>44</v>
@@ -4905,10 +4904,10 @@
         <v>24.4%</v>
       </c>
       <c r="G56">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="H56" t="str">
-        <v>68.9%</v>
+        <v>75.6%</v>
       </c>
       <c r="I56">
         <v>20</v>
@@ -4969,10 +4968,10 @@
         <v>43.5%</v>
       </c>
       <c r="G58">
-        <v>9</v>
+        <v>13</v>
       </c>
       <c r="H58" t="str">
-        <v>39.1%</v>
+        <v>56.5%</v>
       </c>
       <c r="I58">
         <v>0</v>
@@ -5001,10 +5000,10 @@
         <v>0.0%</v>
       </c>
       <c r="G59">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="H59" t="str">
-        <v>88.9%</v>
+        <v>100.0%</v>
       </c>
       <c r="I59">
         <v>10</v>
@@ -5033,10 +5032,10 @@
         <v>2.2%</v>
       </c>
       <c r="G60">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="H60" t="str">
-        <v>95.6%</v>
+        <v>97.8%</v>
       </c>
       <c r="I60">
         <v>22</v>
@@ -5065,10 +5064,10 @@
         <v>3.2%</v>
       </c>
       <c r="G61">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="H61" t="str">
-        <v>87.1%</v>
+        <v>96.8%</v>
       </c>
       <c r="I61">
         <v>6</v>
@@ -5097,10 +5096,10 @@
         <v>17.4%</v>
       </c>
       <c r="G62">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="H62" t="str">
-        <v>73.9%</v>
+        <v>82.6%</v>
       </c>
       <c r="I62">
         <v>4</v>
@@ -5129,10 +5128,10 @@
         <v>5.6%</v>
       </c>
       <c r="G63">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="H63" t="str">
-        <v>88.9%</v>
+        <v>94.4%</v>
       </c>
       <c r="I63">
         <v>6</v>
@@ -5161,10 +5160,10 @@
         <v>17.8%</v>
       </c>
       <c r="G64">
-        <v>30</v>
+        <v>37</v>
       </c>
       <c r="H64" t="str">
-        <v>66.7%</v>
+        <v>82.2%</v>
       </c>
       <c r="I64">
         <v>20</v>
@@ -5193,10 +5192,10 @@
         <v>15.6%</v>
       </c>
       <c r="G65">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="H65" t="str">
-        <v>78.1%</v>
+        <v>84.4%</v>
       </c>
       <c r="I65">
         <v>15</v>
@@ -5225,10 +5224,10 @@
         <v>26.1%</v>
       </c>
       <c r="G66">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="H66" t="str">
-        <v>52.2%</v>
+        <v>73.9%</v>
       </c>
       <c r="I66">
         <v>3</v>
@@ -5257,10 +5256,10 @@
         <v>16.7%</v>
       </c>
       <c r="G67">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="H67" t="str">
-        <v>72.2%</v>
+        <v>83.3%</v>
       </c>
       <c r="I67">
         <v>6</v>
@@ -5289,10 +5288,10 @@
         <v>14.2%</v>
       </c>
       <c r="G68">
-        <v>270</v>
+        <v>302</v>
       </c>
       <c r="H68" t="str">
-        <v>76.7%</v>
+        <v>85.8%</v>
       </c>
       <c r="I68">
         <v>132</v>
@@ -5315,16 +5314,16 @@
         <v>2095</v>
       </c>
       <c r="E70">
-        <v>310</v>
+        <v>243</v>
       </c>
       <c r="F70" t="str">
-        <v>14.8%</v>
+        <v>11.6%</v>
       </c>
       <c r="G70">
-        <v>1568</v>
+        <v>1785</v>
       </c>
       <c r="H70" t="str">
-        <v>74.8%</v>
+        <v>85.2%</v>
       </c>
       <c r="I70">
         <v>838</v>
@@ -5411,10 +5410,10 @@
         <v>20.9%</v>
       </c>
       <c r="G6">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="H6" t="str">
-        <v>72.1%</v>
+        <v>79.1%</v>
       </c>
       <c r="I6">
         <v>13</v>
@@ -5443,10 +5442,10 @@
         <v>82.4%</v>
       </c>
       <c r="G7">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="H7" t="str">
-        <v>5.9%</v>
+        <v>17.6%</v>
       </c>
       <c r="I7">
         <v>0</v>
@@ -5475,10 +5474,10 @@
         <v>17.4%</v>
       </c>
       <c r="G8">
-        <v>27</v>
+        <v>38</v>
       </c>
       <c r="H8" t="str">
-        <v>58.7%</v>
+        <v>82.6%</v>
       </c>
       <c r="I8">
         <v>5</v>
@@ -5507,10 +5506,10 @@
         <v>32.5%</v>
       </c>
       <c r="G9">
-        <v>16</v>
+        <v>27</v>
       </c>
       <c r="H9" t="str">
-        <v>40.0%</v>
+        <v>67.5%</v>
       </c>
       <c r="I9">
         <v>3</v>
@@ -5539,10 +5538,10 @@
         <v>82.4%</v>
       </c>
       <c r="G10">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="H10" t="str">
-        <v>0.0%</v>
+        <v>17.6%</v>
       </c>
       <c r="I10">
         <v>0</v>
@@ -5571,10 +5570,10 @@
         <v>38.6%</v>
       </c>
       <c r="G11">
-        <v>14</v>
+        <v>27</v>
       </c>
       <c r="H11" t="str">
-        <v>31.8%</v>
+        <v>61.4%</v>
       </c>
       <c r="I11">
         <v>0</v>
@@ -5597,16 +5596,16 @@
         <v>43</v>
       </c>
       <c r="E12">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="F12" t="str">
-        <v>34.9%</v>
+        <v>30.2%</v>
       </c>
       <c r="G12">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="H12" t="str">
-        <v>58.1%</v>
+        <v>65.1%</v>
       </c>
       <c r="I12">
         <v>11</v>
@@ -5635,10 +5634,10 @@
         <v>35.3%</v>
       </c>
       <c r="G13">
-        <v>7</v>
+        <v>11</v>
       </c>
       <c r="H13" t="str">
-        <v>41.2%</v>
+        <v>64.7%</v>
       </c>
       <c r="I13">
         <v>3</v>
@@ -5667,10 +5666,10 @@
         <v>26.1%</v>
       </c>
       <c r="G14">
-        <v>22</v>
+        <v>34</v>
       </c>
       <c r="H14" t="str">
-        <v>47.8%</v>
+        <v>73.9%</v>
       </c>
       <c r="I14">
         <v>4</v>
@@ -5795,10 +5794,10 @@
         <v>16.7%</v>
       </c>
       <c r="G18">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="H18" t="str">
-        <v>33.3%</v>
+        <v>83.3%</v>
       </c>
       <c r="I18">
         <v>0</v>
@@ -5891,10 +5890,10 @@
         <v>60.7%</v>
       </c>
       <c r="G21">
-        <v>4</v>
+        <v>11</v>
       </c>
       <c r="H21" t="str">
-        <v>14.3%</v>
+        <v>39.3%</v>
       </c>
       <c r="I21">
         <v>0</v>
@@ -5917,16 +5916,16 @@
         <v>370</v>
       </c>
       <c r="E22">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="F22" t="str">
-        <v>36.5%</v>
+        <v>35.9%</v>
       </c>
       <c r="G22">
-        <v>163</v>
+        <v>235</v>
       </c>
       <c r="H22" t="str">
-        <v>44.1%</v>
+        <v>63.5%</v>
       </c>
       <c r="I22">
         <v>46</v>
@@ -5992,10 +5991,10 @@
         <v>0.0%</v>
       </c>
       <c r="G26">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H26" t="str">
-        <v>85.7%</v>
+        <v>100.0%</v>
       </c>
       <c r="I26">
         <v>4</v>
@@ -6024,10 +6023,10 @@
         <v>18.2%</v>
       </c>
       <c r="G27">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="H27" t="str">
-        <v>45.5%</v>
+        <v>81.8%</v>
       </c>
       <c r="I27">
         <v>2</v>
@@ -6056,10 +6055,10 @@
         <v>0.0%</v>
       </c>
       <c r="G28">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H28" t="str">
-        <v>85.7%</v>
+        <v>100.0%</v>
       </c>
       <c r="I28">
         <v>5</v>
@@ -6088,10 +6087,10 @@
         <v>0.0%</v>
       </c>
       <c r="G29">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H29" t="str">
-        <v>85.7%</v>
+        <v>100.0%</v>
       </c>
       <c r="I29">
         <v>2</v>
@@ -6120,10 +6119,10 @@
         <v>27.3%</v>
       </c>
       <c r="G30">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="H30" t="str">
-        <v>63.6%</v>
+        <v>72.7%</v>
       </c>
       <c r="I30">
         <v>1</v>
@@ -6152,10 +6151,10 @@
         <v>28.6%</v>
       </c>
       <c r="G31">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H31" t="str">
-        <v>57.1%</v>
+        <v>71.4%</v>
       </c>
       <c r="I31">
         <v>0</v>
@@ -6184,10 +6183,10 @@
         <v>0.0%</v>
       </c>
       <c r="G32">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H32" t="str">
-        <v>85.7%</v>
+        <v>100.0%</v>
       </c>
       <c r="I32">
         <v>2</v>
@@ -6248,10 +6247,10 @@
         <v>0.0%</v>
       </c>
       <c r="G34">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H34" t="str">
-        <v>85.7%</v>
+        <v>100.0%</v>
       </c>
       <c r="I34">
         <v>4</v>
@@ -6344,10 +6343,10 @@
         <v>0.0%</v>
       </c>
       <c r="G37">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H37" t="str">
-        <v>50.0%</v>
+        <v>100.0%</v>
       </c>
       <c r="I37">
         <v>0</v>
@@ -6408,10 +6407,10 @@
         <v>9.6%</v>
       </c>
       <c r="G39">
-        <v>63</v>
+        <v>75</v>
       </c>
       <c r="H39" t="str">
-        <v>75.9%</v>
+        <v>90.4%</v>
       </c>
       <c r="I39">
         <v>28</v>
@@ -6477,10 +6476,10 @@
         <v>80.0%</v>
       </c>
       <c r="G43">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H43" t="str">
-        <v>10.0%</v>
+        <v>20.0%</v>
       </c>
       <c r="I43">
         <v>0</v>
@@ -6509,10 +6508,10 @@
         <v>14.3%</v>
       </c>
       <c r="G44">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H44" t="str">
-        <v>71.4%</v>
+        <v>85.7%</v>
       </c>
       <c r="I44">
         <v>0</v>
@@ -6541,10 +6540,10 @@
         <v>55.6%</v>
       </c>
       <c r="G45">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="H45" t="str">
-        <v>11.1%</v>
+        <v>44.4%</v>
       </c>
       <c r="I45">
         <v>1</v>
@@ -6573,10 +6572,10 @@
         <v>57.1%</v>
       </c>
       <c r="G46">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H46" t="str">
-        <v>28.6%</v>
+        <v>42.9%</v>
       </c>
       <c r="I46">
         <v>0</v>
@@ -6637,10 +6636,10 @@
         <v>42.9%</v>
       </c>
       <c r="G48">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H48" t="str">
-        <v>42.9%</v>
+        <v>57.1%</v>
       </c>
       <c r="I48">
         <v>0</v>
@@ -6733,10 +6732,10 @@
         <v>56.4%</v>
       </c>
       <c r="G51">
-        <v>17</v>
+        <v>24</v>
       </c>
       <c r="H51" t="str">
-        <v>30.9%</v>
+        <v>43.6%</v>
       </c>
       <c r="I51">
         <v>2</v>
@@ -6759,16 +6758,16 @@
         <v>508</v>
       </c>
       <c r="E53">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="F53" t="str">
-        <v>34.3%</v>
+        <v>33.9%</v>
       </c>
       <c r="G53">
-        <v>243</v>
+        <v>334</v>
       </c>
       <c r="H53" t="str">
-        <v>47.8%</v>
+        <v>65.7%</v>
       </c>
       <c r="I53">
         <v>76</v>
@@ -6786,342 +6785,6 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K12"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="str">
-        <v>THỐNG KÊ CHI TIẾT 7 MÔN TỰ CHỌN KHỐI 12 THEO CƠ SỞ (NGOÀI TOÁN - VĂN - ANH)</v>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="str">
-        <v>* Áp dụng cho học sinh Khối 12 làm bài khảo sát định hướng tốt nghiệp THPT theo tổ hợp môn</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="str">
-        <v>STT</v>
-      </c>
-      <c r="B4" t="str">
-        <v>Cơ sở</v>
-      </c>
-      <c r="C4" t="str">
-        <v>Môn học tự chọn</v>
-      </c>
-      <c r="D4" t="str">
-        <v>Khối lớp</v>
-      </c>
-      <c r="E4" t="str">
-        <v>Số HS khảo sát</v>
-      </c>
-      <c r="F4" t="str">
-        <v>Điểm dưới TB (&lt; 5.0)</v>
-      </c>
-      <c r="G4" t="str">
-        <v>Tỷ lệ &lt; 5.0</v>
-      </c>
-      <c r="H4" t="str">
-        <v>Điểm Chuẩn (≥ 5.0)</v>
-      </c>
-      <c r="I4" t="str">
-        <v>Tỷ lệ Đạt chuẩn</v>
-      </c>
-      <c r="J4" t="str">
-        <v>Điểm 8 đến 10 (Giỏi)</v>
-      </c>
-      <c r="K4" t="str">
-        <v>Tỷ lệ Giỏi</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5">
-        <v>1</v>
-      </c>
-      <c r="B5" t="str">
-        <v>CS1</v>
-      </c>
-      <c r="C5" t="str">
-        <v>Vật lí</v>
-      </c>
-      <c r="D5" t="str">
-        <v>Khối 12</v>
-      </c>
-      <c r="E5">
-        <v>13</v>
-      </c>
-      <c r="F5">
-        <v>2</v>
-      </c>
-      <c r="G5" t="str">
-        <v>15.4%</v>
-      </c>
-      <c r="H5">
-        <v>11</v>
-      </c>
-      <c r="I5" t="str">
-        <v>84.6%</v>
-      </c>
-      <c r="J5">
-        <v>2</v>
-      </c>
-      <c r="K5" t="str">
-        <v>15.4%</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6">
-        <v>2</v>
-      </c>
-      <c r="B6" t="str">
-        <v>CS1</v>
-      </c>
-      <c r="C6" t="str">
-        <v>Hóa học</v>
-      </c>
-      <c r="D6" t="str">
-        <v>Khối 12</v>
-      </c>
-      <c r="E6">
-        <v>11</v>
-      </c>
-      <c r="F6">
-        <v>4</v>
-      </c>
-      <c r="G6" t="str">
-        <v>36.4%</v>
-      </c>
-      <c r="H6">
-        <v>7</v>
-      </c>
-      <c r="I6" t="str">
-        <v>63.6%</v>
-      </c>
-      <c r="J6">
-        <v>2</v>
-      </c>
-      <c r="K6" t="str">
-        <v>18.2%</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7">
-        <v>3</v>
-      </c>
-      <c r="B7" t="str">
-        <v>CS1</v>
-      </c>
-      <c r="C7" t="str">
-        <v>Sinh học</v>
-      </c>
-      <c r="D7" t="str">
-        <v>Khối 12</v>
-      </c>
-      <c r="E7">
-        <v>10</v>
-      </c>
-      <c r="F7">
-        <v>0</v>
-      </c>
-      <c r="G7" t="str">
-        <v>0.0%</v>
-      </c>
-      <c r="H7">
-        <v>10</v>
-      </c>
-      <c r="I7" t="str">
-        <v>100.0%</v>
-      </c>
-      <c r="J7">
-        <v>3</v>
-      </c>
-      <c r="K7" t="str">
-        <v>30.0%</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8">
-        <v>4</v>
-      </c>
-      <c r="B8" t="str">
-        <v>CS1</v>
-      </c>
-      <c r="C8" t="str">
-        <v>Lịch sử</v>
-      </c>
-      <c r="D8" t="str">
-        <v>Khối 12</v>
-      </c>
-      <c r="E8">
-        <v>11</v>
-      </c>
-      <c r="F8">
-        <v>5</v>
-      </c>
-      <c r="G8" t="str">
-        <v>45.5%</v>
-      </c>
-      <c r="H8">
-        <v>6</v>
-      </c>
-      <c r="I8" t="str">
-        <v>54.5%</v>
-      </c>
-      <c r="J8">
-        <v>0</v>
-      </c>
-      <c r="K8" t="str">
-        <v>0.0%</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9">
-        <v>5</v>
-      </c>
-      <c r="B9" t="str">
-        <v>CS1</v>
-      </c>
-      <c r="C9" t="str">
-        <v>Địa lí</v>
-      </c>
-      <c r="D9" t="str">
-        <v>Khối 12</v>
-      </c>
-      <c r="E9">
-        <v>11</v>
-      </c>
-      <c r="F9">
-        <v>0</v>
-      </c>
-      <c r="G9" t="str">
-        <v>0.0%</v>
-      </c>
-      <c r="H9">
-        <v>11</v>
-      </c>
-      <c r="I9" t="str">
-        <v>100.0%</v>
-      </c>
-      <c r="J9">
-        <v>2</v>
-      </c>
-      <c r="K9" t="str">
-        <v>18.2%</v>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10">
-        <v>6</v>
-      </c>
-      <c r="B10" t="str">
-        <v>CS1</v>
-      </c>
-      <c r="C10" t="str">
-        <v>GD Kinh tế &amp; Pháp luật</v>
-      </c>
-      <c r="D10" t="str">
-        <v>Khối 12</v>
-      </c>
-      <c r="E10">
-        <v>11</v>
-      </c>
-      <c r="F10">
-        <v>0</v>
-      </c>
-      <c r="G10" t="str">
-        <v>0.0%</v>
-      </c>
-      <c r="H10">
-        <v>11</v>
-      </c>
-      <c r="I10" t="str">
-        <v>100.0%</v>
-      </c>
-      <c r="J10">
-        <v>3</v>
-      </c>
-      <c r="K10" t="str">
-        <v>27.3%</v>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11">
-        <v>7</v>
-      </c>
-      <c r="B11" t="str">
-        <v>CS1</v>
-      </c>
-      <c r="C11" t="str">
-        <v>Tin học / ICT</v>
-      </c>
-      <c r="D11" t="str">
-        <v>Khối 12</v>
-      </c>
-      <c r="E11">
-        <v>4</v>
-      </c>
-      <c r="F11">
-        <v>1</v>
-      </c>
-      <c r="G11" t="str">
-        <v>25.0%</v>
-      </c>
-      <c r="H11">
-        <v>3</v>
-      </c>
-      <c r="I11" t="str">
-        <v>75.0%</v>
-      </c>
-      <c r="J11">
-        <v>0</v>
-      </c>
-      <c r="K11" t="str">
-        <v>0.0%</v>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="str">
-        <v>-</v>
-      </c>
-      <c r="B12" t="str">
-        <v>CS1</v>
-      </c>
-      <c r="C12" t="str">
-        <v>TỔNG 7 MÔN TỰ CHỌN K12</v>
-      </c>
-      <c r="D12" t="str">
-        <v>Khối 12</v>
-      </c>
-      <c r="E12">
-        <v>71</v>
-      </c>
-      <c r="F12">
-        <v>12</v>
-      </c>
-      <c r="G12" t="str">
-        <v>16.9%</v>
-      </c>
-      <c r="H12">
-        <v>59</v>
-      </c>
-      <c r="I12" t="str">
-        <v>83.1%</v>
-      </c>
-      <c r="J12">
-        <v>12</v>
-      </c>
-      <c r="K12" t="str">
-        <v>16.9%</v>
-      </c>
-    </row>
-  </sheetData>
-  <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:K12"/>
-  </ignoredErrors>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:K22"/>
   <sheetData>
     <row r="1">
@@ -7806,7 +7469,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <dimension ref="A1:K81"/>
   <sheetData>

</xml_diff>